<commit_message>
Reorganize as a docker image
</commit_message>
<xml_diff>
--- a/2_calculated_metrics/reference_corpus_metrics/reference_corpus_overview.xlsx
+++ b/2_calculated_metrics/reference_corpus_metrics/reference_corpus_overview.xlsx
@@ -20,7 +20,10 @@
     <sheet name="Service_Area" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="Audience" sheetId="12" state="visible" r:id="rId12"/>
     <sheet name="Intended_Outcome" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Coding_Confidence" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Evidence_Confidence" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Service_Conditions_Addressed" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="Conceptual_Theme" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="Coding_Confidence" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Year Counts'!$A$1:$C$68</definedName>
@@ -35,7 +38,10 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Service_Area'!$A$1:$E$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Audience'!$A$1:$E$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Intended_Outcome'!$A$1:$E$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'Coding_Confidence'!$A$1:$E$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'Evidence_Confidence'!$A$1:$E$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'Service_Conditions_Addressed'!$A$1:$E$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'Conceptual_Theme'!$A$1:$E$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'Coding_Confidence'!$A$1:$E$3</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -456,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="43" customWidth="1" min="1" max="1"/>
@@ -714,13 +720,52 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
+          <t>Evidence_Confidence</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Service_Conditions_Addressed</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Conceptual_Theme</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
           <t>Coding_Confidence</t>
         </is>
       </c>
-      <c r="B24" t="n">
+      <c r="B27" t="n">
         <v>2</v>
       </c>
-      <c r="C24" t="n">
+      <c r="C27" t="n">
         <v>7201</v>
       </c>
     </row>
@@ -1648,6 +1693,156 @@
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>feature_value</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>article_count</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>total_articles</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>article_pct</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>rank_within_group</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+  </sheetData>
+  <autoFilter ref="A1:E2"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>feature_value</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>article_count</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>total_articles</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>article_pct</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>rank_within_group</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+  </sheetData>
+  <autoFilter ref="A1:E2"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>feature_value</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>article_count</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>total_articles</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>article_pct</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>rank_within_group</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+  </sheetData>
+  <autoFilter ref="A1:E2"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>